<commit_message>
Estudo 153 R01: unidades compactas (2Q 40–45 m², 3Q 50–60 m²) e máximo de unidades
Planta tipo passa a empacotar cada fileira com o máximo de unidades
dentro das faixas de área, com núcleo posicionado entre unidades; busca
por pavimentos x composição x subsolos com verificação de CA, H/8,
distância aos fundos, vagas (Anexo VII), lazer e permeabilidade.
Unidades: E1 48→64, E2 56→66, E3 80, E4 70→98, E5 112, E6 112→120.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QqPzsPVGMGmQhub9SKc1k5
</commit_message>
<xml_diff>
--- a/estudo-153-wisocki/entregaveis/153 MODELO NUMERICO - OPCOES.xlsx
+++ b/estudo-153-wisocki/entregaveis/153 MODELO NUMERICO - OPCOES.xlsx
@@ -671,38 +671,38 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>64</v>
+      </c>
+      <c r="C2" t="n">
         <v>48</v>
       </c>
-      <c r="C2" t="n">
-        <v>36</v>
-      </c>
       <c r="D2" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>1978.92</v>
+        <v>1965.6</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>788.88</v>
+        <v>848</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>0</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="K2" s="4">
         <f>MAX(0,I2-J2)</f>
         <v/>
       </c>
       <c r="L2" s="4" t="n">
-        <v>4167.2</v>
+        <v>4170.4</v>
       </c>
       <c r="M2" s="4" t="n">
         <v>1055.83</v>
@@ -735,38 +735,38 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="C3" t="n">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="D3" t="n">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>2017.16</v>
+        <v>962.9400000000001</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>1385.2</v>
+        <v>2492.6</v>
       </c>
       <c r="H3" s="4" t="n">
         <v>0</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="K3" s="4">
         <f>MAX(0,I3-J3)</f>
         <v/>
       </c>
       <c r="L3" s="4" t="n">
-        <v>4960.5</v>
+        <v>4982.77</v>
       </c>
       <c r="M3" s="4" t="n">
         <v>1055.83</v>
@@ -799,10 +799,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="C4" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="D4" t="n">
         <v>20</v>
@@ -811,26 +811,26 @@
         <v>0</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>2017.16</v>
+        <v>2410.2</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>1385.2</v>
+        <v>1039.8</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>58</v>
+        <v>84</v>
       </c>
       <c r="K4" s="4">
         <f>MAX(0,I4-J4)</f>
         <v/>
       </c>
       <c r="L4" s="4" t="n">
-        <v>4960.5</v>
+        <v>4972.44</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>2111.67</v>
@@ -863,25 +863,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="C5" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>42</v>
+        <v>84</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>1398.88</v>
+        <v>581.42</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>1399.02</v>
+        <v>2216.76</v>
       </c>
       <c r="I5" s="4" t="n">
         <v>44</v>
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>96</v>
+        <v>112</v>
       </c>
       <c r="C6" t="n">
         <v>32</v>
@@ -936,22 +936,22 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>1714.24</v>
+        <v>1324.48</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1713.92</v>
+        <v>2104</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="K6" s="4">
         <f>MAX(0,I6-J6)</f>
@@ -991,38 +991,38 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C7" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>857.12</v>
+        <v>826.2</v>
       </c>
       <c r="G7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>2570.88</v>
+        <v>2624</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="K7" s="4">
         <f>MAX(0,I7-J7)</f>
         <v/>
       </c>
       <c r="L7" s="4" t="n">
-        <v>4961.4</v>
+        <v>4972.44</v>
       </c>
       <c r="M7" s="4" t="n">
         <v>1055.83</v>

</xml_diff>